<commit_message>
added the stocks api update
</commit_message>
<xml_diff>
--- a/googleSheetApiUpdate.xlsx
+++ b/googleSheetApiUpdate.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\singh\Desktop\projects\codfty\Mobulous_Tech\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FAD16BAB-8143-4754-B91F-D2FB594C390A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FADC7238-07DB-48E3-B55A-7E440C4303E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F974C6E5-2D0F-48CC-B9F3-DB4A6872002E}"/>
   </bookViews>
@@ -1027,7 +1027,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1043,8 +1043,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1054,6 +1062,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFB9A59C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1082,10 +1096,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -1093,8 +1108,19 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1465,7 +1491,7 @@
       <c r="E2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="3" t="s">
         <v>14</v>
       </c>
       <c r="G2" s="2" t="s">
@@ -1507,90 +1533,90 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:9" s="5" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E4" s="2" t="s">
+      <c r="C4" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="H4" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="I4" s="4" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E5" s="2" t="s">
+      <c r="C5" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F5" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="G5" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="H5" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="I5" s="4" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
+    <row r="6" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E6" s="2" t="s">
+      <c r="C6" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="G6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="H6" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="I6" s="2" t="s">
+      <c r="I6" s="4" t="s">
         <v>40</v>
       </c>
     </row>
@@ -3481,7 +3507,11 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:I71" xr:uid="{8F4433F2-1FE6-4C83-83F7-5576DB0FF34D}"/>
+  <hyperlinks>
+    <hyperlink ref="F2" r:id="rId1" xr:uid="{301ADF35-6FAF-4264-9960-22B3449ADB94}"/>
+    <hyperlink ref="E6" r:id="rId2" xr:uid="{0080C597-7F2A-42E9-AA2F-B2FE1EA5ACA8}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>